<commit_message>
Updated on 09-19-2023 at 23:57
</commit_message>
<xml_diff>
--- a/dados_full_brasil.xlsx
+++ b/dados_full_brasil.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gustavo\AppData\Local\Temp\scp14777\home\gustavo\Documents\lovo_code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gustavo\AppData\Local\Temp\scp33883\home\gustavo\Documents\lovo_code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AAFD09B-059A-4321-BB5D-F931DFE6F714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B039BA4-3784-46AC-81C0-D4F2A245735D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4157,7 +4157,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4168,6 +4168,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF81ACA6"/>
         <bgColor rgb="FF9999FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -4198,12 +4210,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4586,7 +4601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q1351"/>
+  <dimension ref="A1:T1351"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:17" ht="15" x14ac:dyDescent="0.2">
@@ -9949,2069 +9964,2070 @@
       </c>
     </row>
     <row r="122" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
-        <v>17</v>
-      </c>
-      <c r="B122" t="s">
-        <v>18</v>
-      </c>
-      <c r="C122" t="s">
-        <v>19</v>
-      </c>
-      <c r="D122" t="s">
+      <c r="A122" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D122" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E122">
+      <c r="E122" s="4">
         <v>85380</v>
       </c>
-      <c r="F122">
+      <c r="F122" s="4">
         <v>7218</v>
       </c>
-      <c r="G122">
+      <c r="G122" s="4">
         <v>5126.857</v>
       </c>
-      <c r="H122">
+      <c r="H122" s="4">
         <v>5901</v>
       </c>
-      <c r="I122">
+      <c r="I122" s="4">
         <v>435</v>
       </c>
-      <c r="J122">
+      <c r="J122" s="4">
         <v>369.714</v>
       </c>
-      <c r="K122">
+      <c r="K122" s="4">
         <v>396.53800000000001</v>
       </c>
-      <c r="L122">
+      <c r="L122" s="4">
         <v>33.523000000000003</v>
       </c>
-      <c r="M122">
+      <c r="M122" s="4">
         <v>23.811</v>
       </c>
-      <c r="N122">
+      <c r="N122" s="4">
         <v>27.407</v>
       </c>
-      <c r="O122">
+      <c r="O122" s="4">
         <v>2.02</v>
       </c>
-      <c r="P122">
+      <c r="P122" s="4">
         <v>1.7170000000000001</v>
       </c>
-      <c r="Q122">
+      <c r="Q122" s="4">
         <v>1.47</v>
       </c>
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
-        <v>17</v>
-      </c>
-      <c r="B123" t="s">
-        <v>18</v>
-      </c>
-      <c r="C123" t="s">
-        <v>19</v>
-      </c>
-      <c r="D123" t="s">
+      <c r="A123" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D123" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E123">
+      <c r="E123" s="4">
         <v>91589</v>
       </c>
-      <c r="F123">
+      <c r="F123" s="4">
         <v>6209</v>
       </c>
-      <c r="G123">
+      <c r="G123" s="4">
         <v>5513.4290000000001</v>
       </c>
-      <c r="H123">
+      <c r="H123" s="4">
         <v>6329</v>
       </c>
-      <c r="I123">
+      <c r="I123" s="4">
         <v>428</v>
       </c>
-      <c r="J123">
+      <c r="J123" s="4">
         <v>379.85700000000003</v>
       </c>
-      <c r="K123">
+      <c r="K123" s="4">
         <v>425.375</v>
       </c>
-      <c r="L123">
+      <c r="L123" s="4">
         <v>28.837</v>
       </c>
-      <c r="M123">
+      <c r="M123" s="4">
         <v>25.606999999999999</v>
       </c>
-      <c r="N123">
+      <c r="N123" s="4">
         <v>29.393999999999998</v>
       </c>
-      <c r="O123">
+      <c r="O123" s="4">
         <v>1.988</v>
       </c>
-      <c r="P123">
+      <c r="P123" s="4">
         <v>1.764</v>
       </c>
-      <c r="Q123">
+      <c r="Q123" s="4">
         <v>1.46</v>
       </c>
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
-        <v>17</v>
-      </c>
-      <c r="B124" t="s">
-        <v>18</v>
-      </c>
-      <c r="C124" t="s">
-        <v>19</v>
-      </c>
-      <c r="D124" t="s">
+      <c r="A124" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D124" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E124">
+      <c r="E124" s="4">
         <v>96559</v>
       </c>
-      <c r="F124">
+      <c r="F124" s="4">
         <v>4970</v>
       </c>
-      <c r="G124">
+      <c r="G124" s="4">
         <v>5435.7139999999999</v>
       </c>
-      <c r="H124">
+      <c r="H124" s="4">
         <v>6750</v>
       </c>
-      <c r="I124">
+      <c r="I124" s="4">
         <v>421</v>
       </c>
-      <c r="J124">
+      <c r="J124" s="4">
         <v>390.57100000000003</v>
       </c>
-      <c r="K124">
+      <c r="K124" s="4">
         <v>448.45800000000003</v>
       </c>
-      <c r="L124">
+      <c r="L124" s="4">
         <v>23.082999999999998</v>
       </c>
-      <c r="M124">
+      <c r="M124" s="4">
         <v>25.245999999999999</v>
       </c>
-      <c r="N124">
+      <c r="N124" s="4">
         <v>31.35</v>
       </c>
-      <c r="O124">
+      <c r="O124" s="4">
         <v>1.9550000000000001</v>
       </c>
-      <c r="P124">
+      <c r="P124" s="4">
         <v>1.8140000000000001</v>
       </c>
-      <c r="Q124">
+      <c r="Q124" s="4">
         <v>1.45</v>
       </c>
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
-        <v>17</v>
-      </c>
-      <c r="B125" t="s">
-        <v>18</v>
-      </c>
-      <c r="C125" t="s">
-        <v>19</v>
-      </c>
-      <c r="D125" t="s">
+      <c r="A125" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D125" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E125">
+      <c r="E125" s="4">
         <v>101147</v>
       </c>
-      <c r="F125">
+      <c r="F125" s="4">
         <v>4588</v>
       </c>
-      <c r="G125">
+      <c r="G125" s="4">
         <v>5608.4290000000001</v>
       </c>
-      <c r="H125">
+      <c r="H125" s="4">
         <v>7025</v>
       </c>
-      <c r="I125">
+      <c r="I125" s="4">
         <v>275</v>
       </c>
-      <c r="J125">
+      <c r="J125" s="4">
         <v>402.85700000000003</v>
       </c>
-      <c r="K125">
+      <c r="K125" s="4">
         <v>469.76600000000002</v>
       </c>
-      <c r="L125">
+      <c r="L125" s="4">
         <v>21.308</v>
       </c>
-      <c r="M125">
+      <c r="M125" s="4">
         <v>26.047999999999998</v>
       </c>
-      <c r="N125">
+      <c r="N125" s="4">
         <v>32.627000000000002</v>
       </c>
-      <c r="O125">
+      <c r="O125" s="4">
         <v>1.2769999999999999</v>
       </c>
-      <c r="P125">
+      <c r="P125" s="4">
         <v>1.871</v>
       </c>
-      <c r="Q125">
+      <c r="Q125" s="4">
         <v>1.45</v>
       </c>
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
-        <v>17</v>
-      </c>
-      <c r="B126" t="s">
-        <v>18</v>
-      </c>
-      <c r="C126" t="s">
-        <v>19</v>
-      </c>
-      <c r="D126" t="s">
+      <c r="A126" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D126" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E126">
+      <c r="E126" s="4">
         <v>107780</v>
       </c>
-      <c r="F126">
+      <c r="F126" s="4">
         <v>6633</v>
       </c>
-      <c r="G126">
+      <c r="G126" s="4">
         <v>5897</v>
       </c>
-      <c r="H126">
+      <c r="H126" s="4">
         <v>7321</v>
       </c>
-      <c r="I126">
+      <c r="I126" s="4">
         <v>296</v>
       </c>
-      <c r="J126">
+      <c r="J126" s="4">
         <v>396.85700000000003</v>
       </c>
-      <c r="K126">
+      <c r="K126" s="4">
         <v>500.572</v>
       </c>
-      <c r="L126">
+      <c r="L126" s="4">
         <v>30.806000000000001</v>
       </c>
-      <c r="M126">
+      <c r="M126" s="4">
         <v>27.388000000000002</v>
       </c>
-      <c r="N126">
+      <c r="N126" s="4">
         <v>34.002000000000002</v>
       </c>
-      <c r="O126">
+      <c r="O126" s="4">
         <v>1.375</v>
       </c>
-      <c r="P126">
+      <c r="P126" s="4">
         <v>1.843</v>
       </c>
-      <c r="Q126">
+      <c r="Q126" s="4">
         <v>1.44</v>
       </c>
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>17</v>
-      </c>
-      <c r="B127" t="s">
-        <v>18</v>
-      </c>
-      <c r="C127" t="s">
-        <v>19</v>
-      </c>
-      <c r="D127" t="s">
+      <c r="A127" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D127" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="E127">
+      <c r="E127" s="4">
         <v>114715</v>
       </c>
-      <c r="F127">
+      <c r="F127" s="4">
         <v>6935</v>
       </c>
-      <c r="G127">
+      <c r="G127" s="4">
         <v>6118.4290000000001</v>
       </c>
-      <c r="H127">
+      <c r="H127" s="4">
         <v>7921</v>
       </c>
-      <c r="I127">
+      <c r="I127" s="4">
         <v>600</v>
       </c>
-      <c r="J127">
+      <c r="J127" s="4">
         <v>414.85700000000003</v>
       </c>
-      <c r="K127">
+      <c r="K127" s="4">
         <v>532.78099999999995</v>
       </c>
-      <c r="L127">
+      <c r="L127" s="4">
         <v>32.209000000000003</v>
       </c>
-      <c r="M127">
+      <c r="M127" s="4">
         <v>28.416</v>
       </c>
-      <c r="N127">
+      <c r="N127" s="4">
         <v>36.787999999999997</v>
       </c>
-      <c r="O127">
+      <c r="O127" s="4">
         <v>2.7869999999999999</v>
       </c>
-      <c r="P127">
+      <c r="P127" s="4">
         <v>1.927</v>
       </c>
-      <c r="Q127">
+      <c r="Q127" s="4">
         <v>1.43</v>
       </c>
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
-        <v>17</v>
-      </c>
-      <c r="B128" t="s">
-        <v>18</v>
-      </c>
-      <c r="C128" t="s">
-        <v>19</v>
-      </c>
-      <c r="D128" t="s">
+      <c r="A128" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D128" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E128">
+      <c r="E128" s="4">
         <v>125218</v>
       </c>
-      <c r="F128">
+      <c r="F128" s="4">
         <v>10503</v>
       </c>
-      <c r="G128">
+      <c r="G128" s="4">
         <v>6722.2860000000001</v>
       </c>
-      <c r="H128">
+      <c r="H128" s="4">
         <v>8536</v>
       </c>
-      <c r="I128">
+      <c r="I128" s="4">
         <v>615</v>
       </c>
-      <c r="J128">
+      <c r="J128" s="4">
         <v>438.57100000000003</v>
       </c>
-      <c r="K128">
+      <c r="K128" s="4">
         <v>581.56100000000004</v>
       </c>
-      <c r="L128">
+      <c r="L128" s="4">
         <v>48.78</v>
       </c>
-      <c r="M128">
+      <c r="M128" s="4">
         <v>31.221</v>
       </c>
-      <c r="N128">
+      <c r="N128" s="4">
         <v>39.645000000000003</v>
       </c>
-      <c r="O128">
+      <c r="O128" s="4">
         <v>2.8559999999999999</v>
       </c>
-      <c r="P128">
+      <c r="P128" s="4">
         <v>2.0369999999999999</v>
       </c>
-      <c r="Q128">
+      <c r="Q128" s="4">
         <v>1.43</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
-        <v>17</v>
-      </c>
-      <c r="B129" t="s">
-        <v>18</v>
-      </c>
-      <c r="C129" t="s">
-        <v>19</v>
-      </c>
-      <c r="D129" t="s">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A129" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D129" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E129">
+      <c r="E129" s="4">
         <v>135106</v>
       </c>
-      <c r="F129">
+      <c r="F129" s="4">
         <v>9888</v>
       </c>
-      <c r="G129">
+      <c r="G129" s="4">
         <v>7103.7139999999999</v>
       </c>
-      <c r="H129">
+      <c r="H129" s="4">
         <v>9146</v>
       </c>
-      <c r="I129">
+      <c r="I129" s="4">
         <v>610</v>
       </c>
-      <c r="J129">
+      <c r="J129" s="4">
         <v>463.57100000000003</v>
       </c>
-      <c r="K129">
+      <c r="K129" s="4">
         <v>627.48500000000001</v>
       </c>
-      <c r="L129">
+      <c r="L129" s="4">
         <v>45.923999999999999</v>
       </c>
-      <c r="M129">
+      <c r="M129" s="4">
         <v>32.991999999999997</v>
       </c>
-      <c r="N129">
+      <c r="N129" s="4">
         <v>42.478000000000002</v>
       </c>
-      <c r="O129">
+      <c r="O129" s="4">
         <v>2.8330000000000002</v>
       </c>
-      <c r="P129">
+      <c r="P129" s="4">
         <v>2.153</v>
       </c>
-      <c r="Q129">
+      <c r="Q129" s="4">
         <v>1.42</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
-        <v>17</v>
-      </c>
-      <c r="B130" t="s">
-        <v>18</v>
-      </c>
-      <c r="C130" t="s">
-        <v>19</v>
-      </c>
-      <c r="D130" t="s">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A130" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D130" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E130">
+      <c r="E130" s="4">
         <v>145328</v>
       </c>
-      <c r="F130">
+      <c r="F130" s="4">
         <v>10222</v>
       </c>
-      <c r="G130">
+      <c r="G130" s="4">
         <v>7677</v>
       </c>
-      <c r="H130">
+      <c r="H130" s="4">
         <v>9897</v>
       </c>
-      <c r="I130">
+      <c r="I130" s="4">
         <v>751</v>
       </c>
-      <c r="J130">
+      <c r="J130" s="4">
         <v>509.714</v>
       </c>
-      <c r="K130">
+      <c r="K130" s="4">
         <v>674.96</v>
       </c>
-      <c r="L130">
+      <c r="L130" s="4">
         <v>47.475000000000001</v>
       </c>
-      <c r="M130">
+      <c r="M130" s="4">
         <v>35.655000000000001</v>
       </c>
-      <c r="N130">
+      <c r="N130" s="4">
         <v>45.966000000000001</v>
       </c>
-      <c r="O130">
+      <c r="O130" s="4">
         <v>3.488</v>
       </c>
-      <c r="P130">
+      <c r="P130" s="4">
         <v>2.367</v>
       </c>
-      <c r="Q130">
+      <c r="Q130" s="4">
         <v>1.41</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
-        <v>17</v>
-      </c>
-      <c r="B131" t="s">
-        <v>18</v>
-      </c>
-      <c r="C131" t="s">
-        <v>19</v>
-      </c>
-      <c r="D131" t="s">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A131" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D131" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E131">
+      <c r="E131" s="4">
         <v>155939</v>
       </c>
-      <c r="F131">
+      <c r="F131" s="4">
         <v>10611</v>
       </c>
-      <c r="G131">
+      <c r="G131" s="4">
         <v>8482.857</v>
       </c>
-      <c r="H131">
+      <c r="H131" s="4">
         <v>10627</v>
       </c>
-      <c r="I131">
+      <c r="I131" s="4">
         <v>730</v>
       </c>
-      <c r="J131">
+      <c r="J131" s="4">
         <v>553.85699999999997</v>
       </c>
-      <c r="K131">
+      <c r="K131" s="4">
         <v>724.24199999999996</v>
       </c>
-      <c r="L131">
+      <c r="L131" s="4">
         <v>49.281999999999996</v>
       </c>
-      <c r="M131">
+      <c r="M131" s="4">
         <v>39.398000000000003</v>
       </c>
-      <c r="N131">
+      <c r="N131" s="4">
         <v>49.356000000000002</v>
       </c>
-      <c r="O131">
+      <c r="O131" s="4">
         <v>3.39</v>
       </c>
-      <c r="P131">
+      <c r="P131" s="4">
         <v>2.5720000000000001</v>
       </c>
-      <c r="Q131">
+      <c r="Q131" s="4">
         <v>1.4</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
-        <v>17</v>
-      </c>
-      <c r="B132" t="s">
-        <v>18</v>
-      </c>
-      <c r="C132" t="s">
-        <v>19</v>
-      </c>
-      <c r="D132" t="s">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A132" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D132" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E132">
+      <c r="E132" s="4">
         <v>162699</v>
       </c>
-      <c r="F132">
+      <c r="F132" s="4">
         <v>6760</v>
       </c>
-      <c r="G132">
+      <c r="G132" s="4">
         <v>8793.143</v>
       </c>
-      <c r="H132">
+      <c r="H132" s="4">
         <v>11123</v>
       </c>
-      <c r="I132">
+      <c r="I132" s="4">
         <v>496</v>
       </c>
-      <c r="J132">
+      <c r="J132" s="4">
         <v>585.42899999999997</v>
       </c>
-      <c r="K132">
+      <c r="K132" s="4">
         <v>755.63800000000003</v>
       </c>
-      <c r="L132">
+      <c r="L132" s="4">
         <v>31.396000000000001</v>
       </c>
-      <c r="M132">
+      <c r="M132" s="4">
         <v>40.838999999999999</v>
       </c>
-      <c r="N132">
+      <c r="N132" s="4">
         <v>51.66</v>
       </c>
-      <c r="O132">
+      <c r="O132" s="4">
         <v>2.3039999999999998</v>
       </c>
-      <c r="P132">
+      <c r="P132" s="4">
         <v>2.7189999999999999</v>
       </c>
-      <c r="Q132">
+      <c r="Q132" s="4">
         <v>1.39</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
-        <v>17</v>
-      </c>
-      <c r="B133" t="s">
-        <v>18</v>
-      </c>
-      <c r="C133" t="s">
-        <v>19</v>
-      </c>
-      <c r="D133" t="s">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A133" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D133" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E133">
+      <c r="E133" s="4">
         <v>168331</v>
       </c>
-      <c r="F133">
+      <c r="F133" s="4">
         <v>5632</v>
       </c>
-      <c r="G133">
+      <c r="G133" s="4">
         <v>8650.143</v>
       </c>
-      <c r="H133">
+      <c r="H133" s="4">
         <v>11519</v>
       </c>
-      <c r="I133">
+      <c r="I133" s="4">
         <v>396</v>
       </c>
-      <c r="J133">
+      <c r="J133" s="4">
         <v>599.71400000000006</v>
       </c>
-      <c r="K133">
+      <c r="K133" s="4">
         <v>781.79499999999996</v>
       </c>
-      <c r="L133">
+      <c r="L133" s="4">
         <v>26.157</v>
       </c>
-      <c r="M133">
+      <c r="M133" s="4">
         <v>40.174999999999997</v>
       </c>
-      <c r="N133">
+      <c r="N133" s="4">
         <v>53.499000000000002</v>
       </c>
-      <c r="O133">
+      <c r="O133" s="4">
         <v>1.839</v>
       </c>
-      <c r="P133">
+      <c r="P133" s="4">
         <v>2.7850000000000001</v>
       </c>
-      <c r="Q133">
+      <c r="Q133" s="4">
         <v>1.39</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A134" t="s">
-        <v>17</v>
-      </c>
-      <c r="B134" t="s">
-        <v>18</v>
-      </c>
-      <c r="C134" t="s">
-        <v>19</v>
-      </c>
-      <c r="D134" t="s">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A134" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D134" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E134">
+      <c r="E134" s="4">
         <v>177589</v>
       </c>
-      <c r="F134">
+      <c r="F134" s="4">
         <v>9258</v>
       </c>
-      <c r="G134">
+      <c r="G134" s="4">
         <v>8982</v>
       </c>
-      <c r="H134">
+      <c r="H134" s="4">
         <v>12400</v>
       </c>
-      <c r="I134">
+      <c r="I134" s="4">
         <v>881</v>
       </c>
-      <c r="J134">
+      <c r="J134" s="4">
         <v>639.85699999999997</v>
       </c>
-      <c r="K134">
+      <c r="K134" s="4">
         <v>824.79300000000001</v>
       </c>
-      <c r="L134">
+      <c r="L134" s="4">
         <v>42.997999999999998</v>
       </c>
-      <c r="M134">
+      <c r="M134" s="4">
         <v>41.716000000000001</v>
       </c>
-      <c r="N134">
+      <c r="N134" s="4">
         <v>57.59</v>
       </c>
-      <c r="O134">
+      <c r="O134" s="4">
         <v>4.0919999999999996</v>
       </c>
-      <c r="P134">
+      <c r="P134" s="4">
         <v>2.972</v>
       </c>
-      <c r="Q134">
+      <c r="Q134" s="4">
         <v>1.39</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
-        <v>17</v>
-      </c>
-      <c r="B135" t="s">
-        <v>18</v>
-      </c>
-      <c r="C135" t="s">
-        <v>19</v>
-      </c>
-      <c r="D135" t="s">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A135" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D135" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="E135">
+      <c r="E135" s="4">
         <v>188974</v>
       </c>
-      <c r="F135">
+      <c r="F135" s="4">
         <v>11385</v>
       </c>
-      <c r="G135">
+      <c r="G135" s="4">
         <v>9108</v>
       </c>
-      <c r="H135">
+      <c r="H135" s="4">
         <v>13149</v>
       </c>
-      <c r="I135">
+      <c r="I135" s="4">
         <v>749</v>
       </c>
-      <c r="J135">
+      <c r="J135" s="4">
         <v>659</v>
       </c>
-      <c r="K135">
+      <c r="K135" s="4">
         <v>877.66899999999998</v>
       </c>
-      <c r="L135">
+      <c r="L135" s="4">
         <v>52.875999999999998</v>
       </c>
-      <c r="M135">
+      <c r="M135" s="4">
         <v>42.301000000000002</v>
       </c>
-      <c r="N135">
+      <c r="N135" s="4">
         <v>61.069000000000003</v>
       </c>
-      <c r="O135">
+      <c r="O135" s="4">
         <v>3.4790000000000001</v>
       </c>
-      <c r="P135">
+      <c r="P135" s="4">
         <v>3.0609999999999999</v>
       </c>
-      <c r="Q135">
+      <c r="Q135" s="4">
         <v>1.38</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
-        <v>17</v>
-      </c>
-      <c r="B136" t="s">
-        <v>18</v>
-      </c>
-      <c r="C136" t="s">
-        <v>19</v>
-      </c>
-      <c r="D136" t="s">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A136" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D136" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E136">
+      <c r="E136" s="4">
         <v>202918</v>
       </c>
-      <c r="F136">
+      <c r="F136" s="4">
         <v>13944</v>
       </c>
-      <c r="G136">
+      <c r="G136" s="4">
         <v>9687.4290000000001</v>
       </c>
-      <c r="H136">
+      <c r="H136" s="4">
         <v>13993</v>
       </c>
-      <c r="I136">
+      <c r="I136" s="4">
         <v>844</v>
       </c>
-      <c r="J136">
+      <c r="J136" s="4">
         <v>692.42899999999997</v>
       </c>
-      <c r="K136">
+      <c r="K136" s="4">
         <v>942.43</v>
       </c>
-      <c r="L136">
+      <c r="L136" s="4">
         <v>64.760999999999996</v>
       </c>
-      <c r="M136">
+      <c r="M136" s="4">
         <v>44.991999999999997</v>
       </c>
-      <c r="N136">
+      <c r="N136" s="4">
         <v>64.989000000000004</v>
       </c>
-      <c r="O136">
+      <c r="O136" s="4">
         <v>3.92</v>
       </c>
-      <c r="P136">
+      <c r="P136" s="4">
         <v>3.2160000000000002</v>
       </c>
-      <c r="Q136">
+      <c r="Q136" s="4">
         <v>1.38</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
-        <v>17</v>
-      </c>
-      <c r="B137" t="s">
-        <v>18</v>
-      </c>
-      <c r="C137" t="s">
-        <v>19</v>
-      </c>
-      <c r="D137" t="s">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A137" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D137" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E137">
+      <c r="E137" s="4">
         <v>218223</v>
       </c>
-      <c r="F137">
+      <c r="F137" s="4">
         <v>15305</v>
       </c>
-      <c r="G137">
+      <c r="G137" s="4">
         <v>10413.571</v>
       </c>
-      <c r="H137">
+      <c r="H137" s="4">
         <v>14817</v>
       </c>
-      <c r="I137">
+      <c r="I137" s="4">
         <v>824</v>
       </c>
-      <c r="J137">
+      <c r="J137" s="4">
         <v>702.85699999999997</v>
       </c>
-      <c r="K137">
+      <c r="K137" s="4">
         <v>1013.513</v>
       </c>
-      <c r="L137">
+      <c r="L137" s="4">
         <v>71.081999999999994</v>
       </c>
-      <c r="M137">
+      <c r="M137" s="4">
         <v>48.365000000000002</v>
       </c>
-      <c r="N137">
+      <c r="N137" s="4">
         <v>68.816000000000003</v>
       </c>
-      <c r="O137">
+      <c r="O137" s="4">
         <v>3.827</v>
       </c>
-      <c r="P137">
+      <c r="P137" s="4">
         <v>3.2639999999999998</v>
       </c>
-      <c r="Q137">
+      <c r="Q137" s="4">
         <v>1.37</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
-        <v>17</v>
-      </c>
-      <c r="B138" t="s">
-        <v>18</v>
-      </c>
-      <c r="C138" t="s">
-        <v>19</v>
-      </c>
-      <c r="D138" t="s">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A138" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D138" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E138">
+      <c r="E138" s="4">
         <v>233142</v>
       </c>
-      <c r="F138">
+      <c r="F138" s="4">
         <v>14919</v>
       </c>
-      <c r="G138">
+      <c r="G138" s="4">
         <v>11029</v>
       </c>
-      <c r="H138">
+      <c r="H138" s="4">
         <v>15633</v>
       </c>
-      <c r="I138">
+      <c r="I138" s="4">
         <v>816</v>
       </c>
-      <c r="J138">
+      <c r="J138" s="4">
         <v>715.14300000000003</v>
       </c>
-      <c r="K138">
+      <c r="K138" s="4">
         <v>1082.8019999999999</v>
       </c>
-      <c r="L138">
+      <c r="L138" s="4">
         <v>69.290000000000006</v>
       </c>
-      <c r="M138">
+      <c r="M138" s="4">
         <v>51.222999999999999</v>
       </c>
-      <c r="N138">
+      <c r="N138" s="4">
         <v>72.605999999999995</v>
       </c>
-      <c r="O138">
+      <c r="O138" s="4">
         <v>3.79</v>
       </c>
-      <c r="P138">
+      <c r="P138" s="4">
         <v>3.3210000000000002</v>
       </c>
-      <c r="Q138">
+      <c r="Q138" s="4">
         <v>1.37</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
-        <v>17</v>
-      </c>
-      <c r="B139" t="s">
-        <v>18</v>
-      </c>
-      <c r="C139" t="s">
-        <v>19</v>
-      </c>
-      <c r="D139" t="s">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A139" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D139" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E139">
+      <c r="E139" s="4">
         <v>241080</v>
       </c>
-      <c r="F139">
+      <c r="F139" s="4">
         <v>7938</v>
       </c>
-      <c r="G139">
+      <c r="G139" s="4">
         <v>11197.286</v>
       </c>
-      <c r="H139">
+      <c r="H139" s="4">
         <v>16118</v>
       </c>
-      <c r="I139">
+      <c r="I139" s="4">
         <v>485</v>
       </c>
-      <c r="J139">
+      <c r="J139" s="4">
         <v>713.57100000000003</v>
       </c>
-      <c r="K139">
+      <c r="K139" s="4">
         <v>1119.67</v>
       </c>
-      <c r="L139">
+      <c r="L139" s="4">
         <v>36.866999999999997</v>
       </c>
-      <c r="M139">
+      <c r="M139" s="4">
         <v>52.005000000000003</v>
       </c>
-      <c r="N139">
+      <c r="N139" s="4">
         <v>74.858000000000004</v>
       </c>
-      <c r="O139">
+      <c r="O139" s="4">
         <v>2.2530000000000001</v>
       </c>
-      <c r="P139">
+      <c r="P139" s="4">
         <v>3.3140000000000001</v>
       </c>
-      <c r="Q139">
+      <c r="Q139" s="4">
         <v>1.36</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
-        <v>17</v>
-      </c>
-      <c r="B140" t="s">
-        <v>18</v>
-      </c>
-      <c r="C140" t="s">
-        <v>19</v>
-      </c>
-      <c r="D140" t="s">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A140" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D140" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E140">
+      <c r="E140" s="4">
         <v>254220</v>
       </c>
-      <c r="F140">
+      <c r="F140" s="4">
         <v>13140</v>
       </c>
-      <c r="G140">
+      <c r="G140" s="4">
         <v>12269.857</v>
       </c>
-      <c r="H140">
+      <c r="H140" s="4">
         <v>16792</v>
       </c>
-      <c r="I140">
+      <c r="I140" s="4">
         <v>674</v>
       </c>
-      <c r="J140">
+      <c r="J140" s="4">
         <v>753.28599999999994</v>
       </c>
-      <c r="K140">
+      <c r="K140" s="4">
         <v>1180.6969999999999</v>
       </c>
-      <c r="L140">
+      <c r="L140" s="4">
         <v>61.027000000000001</v>
       </c>
-      <c r="M140">
+      <c r="M140" s="4">
         <v>56.985999999999997</v>
       </c>
-      <c r="N140">
+      <c r="N140" s="4">
         <v>77.989000000000004</v>
       </c>
-      <c r="O140">
+      <c r="O140" s="4">
         <v>3.13</v>
       </c>
-      <c r="P140">
+      <c r="P140" s="4">
         <v>3.4990000000000001</v>
       </c>
-      <c r="Q140">
+      <c r="Q140" s="4">
         <v>1.35</v>
       </c>
-    </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A141" t="s">
-        <v>17</v>
-      </c>
-      <c r="B141" t="s">
-        <v>18</v>
-      </c>
-      <c r="C141" t="s">
-        <v>19</v>
-      </c>
-      <c r="D141" t="s">
+      <c r="T140" s="5"/>
+    </row>
+    <row r="141" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A141" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D141" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E141">
+      <c r="E141" s="4">
         <v>271628</v>
       </c>
-      <c r="F141">
+      <c r="F141" s="4">
         <v>17408</v>
       </c>
-      <c r="G141">
+      <c r="G141" s="4">
         <v>13434.143</v>
       </c>
-      <c r="H141">
+      <c r="H141" s="4">
         <v>17971</v>
       </c>
-      <c r="I141">
+      <c r="I141" s="4">
         <v>1179</v>
       </c>
-      <c r="J141">
+      <c r="J141" s="4">
         <v>795.85699999999997</v>
       </c>
-      <c r="K141">
+      <c r="K141" s="4">
         <v>1261.547</v>
       </c>
-      <c r="L141">
+      <c r="L141" s="4">
         <v>80.849999999999994</v>
       </c>
-      <c r="M141">
+      <c r="M141" s="4">
         <v>62.393000000000001</v>
       </c>
-      <c r="N141">
+      <c r="N141" s="4">
         <v>83.463999999999999</v>
       </c>
-      <c r="O141">
+      <c r="O141" s="4">
         <v>5.476</v>
       </c>
-      <c r="P141">
+      <c r="P141" s="4">
         <v>3.6960000000000002</v>
       </c>
-      <c r="Q141">
+      <c r="Q141" s="4">
         <v>1.34</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
-        <v>17</v>
-      </c>
-      <c r="B142" t="s">
-        <v>18</v>
-      </c>
-      <c r="C142" t="s">
-        <v>19</v>
-      </c>
-      <c r="D142" t="s">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A142" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D142" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E142">
+      <c r="E142" s="4">
         <v>291579</v>
       </c>
-      <c r="F142">
+      <c r="F142" s="4">
         <v>19951</v>
       </c>
-      <c r="G142">
+      <c r="G142" s="4">
         <v>14657.857</v>
       </c>
-      <c r="H142">
+      <c r="H142" s="4">
         <v>18859</v>
       </c>
-      <c r="I142">
+      <c r="I142" s="4">
         <v>888</v>
       </c>
-      <c r="J142">
+      <c r="J142" s="4">
         <v>815.71400000000006</v>
       </c>
-      <c r="K142">
+      <c r="K142" s="4">
         <v>1354.2070000000001</v>
       </c>
-      <c r="L142">
+      <c r="L142" s="4">
         <v>92.66</v>
       </c>
-      <c r="M142">
+      <c r="M142" s="4">
         <v>68.076999999999998</v>
       </c>
-      <c r="N142">
+      <c r="N142" s="4">
         <v>87.588999999999999</v>
       </c>
-      <c r="O142">
+      <c r="O142" s="4">
         <v>4.1239999999999997</v>
       </c>
-      <c r="P142">
+      <c r="P142" s="4">
         <v>3.7879999999999998</v>
       </c>
-      <c r="Q142">
+      <c r="Q142" s="4">
         <v>1.33</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
-        <v>17</v>
-      </c>
-      <c r="B143" t="s">
-        <v>18</v>
-      </c>
-      <c r="C143" t="s">
-        <v>19</v>
-      </c>
-      <c r="D143" t="s">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A143" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D143" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E143">
+      <c r="E143" s="4">
         <v>310087</v>
       </c>
-      <c r="F143">
+      <c r="F143" s="4">
         <v>18508</v>
       </c>
-      <c r="G143">
+      <c r="G143" s="4">
         <v>15309.857</v>
       </c>
-      <c r="H143">
+      <c r="H143" s="4">
         <v>20047</v>
       </c>
-      <c r="I143">
+      <c r="I143" s="4">
         <v>1188</v>
       </c>
-      <c r="J143">
+      <c r="J143" s="4">
         <v>864.85699999999997</v>
       </c>
-      <c r="K143">
+      <c r="K143" s="4">
         <v>1440.165</v>
       </c>
-      <c r="L143">
+      <c r="L143" s="4">
         <v>85.957999999999998</v>
       </c>
-      <c r="M143">
+      <c r="M143" s="4">
         <v>71.105000000000004</v>
       </c>
-      <c r="N143">
+      <c r="N143" s="4">
         <v>93.105999999999995</v>
       </c>
-      <c r="O143">
+      <c r="O143" s="4">
         <v>5.5179999999999998</v>
       </c>
-      <c r="P143">
+      <c r="P143" s="4">
         <v>4.0170000000000003</v>
       </c>
-      <c r="Q143">
+      <c r="Q143" s="4">
         <v>1.32</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
-        <v>17</v>
-      </c>
-      <c r="B144" t="s">
-        <v>18</v>
-      </c>
-      <c r="C144" t="s">
-        <v>19</v>
-      </c>
-      <c r="D144" t="s">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A144" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D144" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E144">
+      <c r="E144" s="4">
         <v>330890</v>
       </c>
-      <c r="F144">
+      <c r="F144" s="4">
         <v>20803</v>
       </c>
-      <c r="G144">
+      <c r="G144" s="4">
         <v>16095.286</v>
       </c>
-      <c r="H144">
+      <c r="H144" s="4">
         <v>21048</v>
       </c>
-      <c r="I144">
+      <c r="I144" s="4">
         <v>1001</v>
       </c>
-      <c r="J144">
+      <c r="J144" s="4">
         <v>890.14300000000003</v>
       </c>
-      <c r="K144">
+      <c r="K144" s="4">
         <v>1536.7819999999999</v>
       </c>
-      <c r="L144">
+      <c r="L144" s="4">
         <v>96.617000000000004</v>
       </c>
-      <c r="M144">
+      <c r="M144" s="4">
         <v>74.753</v>
       </c>
-      <c r="N144">
+      <c r="N144" s="4">
         <v>97.754999999999995</v>
       </c>
-      <c r="O144">
+      <c r="O144" s="4">
         <v>4.649</v>
       </c>
-      <c r="P144">
+      <c r="P144" s="4">
         <v>4.1340000000000003</v>
       </c>
-      <c r="Q144">
+      <c r="Q144" s="4">
         <v>1.32</v>
       </c>
     </row>
     <row r="145" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A145" t="s">
-        <v>17</v>
-      </c>
-      <c r="B145" t="s">
-        <v>18</v>
-      </c>
-      <c r="C145" t="s">
-        <v>19</v>
-      </c>
-      <c r="D145" t="s">
+      <c r="A145" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D145" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E145">
+      <c r="E145" s="4">
         <v>347398</v>
       </c>
-      <c r="F145">
+      <c r="F145" s="4">
         <v>16508</v>
       </c>
-      <c r="G145">
+      <c r="G145" s="4">
         <v>16322.286</v>
       </c>
-      <c r="H145">
+      <c r="H145" s="4">
         <v>22013</v>
       </c>
-      <c r="I145">
+      <c r="I145" s="4">
         <v>965</v>
       </c>
-      <c r="J145">
+      <c r="J145" s="4">
         <v>911.42899999999997</v>
       </c>
-      <c r="K145">
+      <c r="K145" s="4">
         <v>1613.452</v>
       </c>
-      <c r="L145">
+      <c r="L145" s="4">
         <v>76.67</v>
       </c>
-      <c r="M145">
+      <c r="M145" s="4">
         <v>75.807000000000002</v>
       </c>
-      <c r="N145">
+      <c r="N145" s="4">
         <v>102.23699999999999</v>
       </c>
-      <c r="O145">
+      <c r="O145" s="4">
         <v>4.4820000000000002</v>
       </c>
-      <c r="P145">
+      <c r="P145" s="4">
         <v>4.2329999999999997</v>
       </c>
-      <c r="Q145">
+      <c r="Q145" s="4">
         <v>1.31</v>
       </c>
     </row>
     <row r="146" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
-        <v>17</v>
-      </c>
-      <c r="B146" t="s">
-        <v>18</v>
-      </c>
-      <c r="C146" t="s">
-        <v>19</v>
-      </c>
-      <c r="D146" t="s">
+      <c r="A146" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C146" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D146" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E146">
+      <c r="E146" s="4">
         <v>363211</v>
       </c>
-      <c r="F146">
+      <c r="F146" s="4">
         <v>15813</v>
       </c>
-      <c r="G146">
+      <c r="G146" s="4">
         <v>17447.286</v>
       </c>
-      <c r="H146">
+      <c r="H146" s="4">
         <v>22666</v>
       </c>
-      <c r="I146">
+      <c r="I146" s="4">
         <v>653</v>
       </c>
-      <c r="J146">
+      <c r="J146" s="4">
         <v>935.42899999999997</v>
       </c>
-      <c r="K146">
+      <c r="K146" s="4">
         <v>1686.894</v>
       </c>
-      <c r="L146">
+      <c r="L146" s="4">
         <v>73.441999999999993</v>
       </c>
-      <c r="M146">
+      <c r="M146" s="4">
         <v>81.031999999999996</v>
       </c>
-      <c r="N146">
+      <c r="N146" s="4">
         <v>105.27</v>
       </c>
-      <c r="O146">
+      <c r="O146" s="4">
         <v>3.0329999999999999</v>
       </c>
-      <c r="P146">
+      <c r="P146" s="4">
         <v>4.3440000000000003</v>
       </c>
-      <c r="Q146">
+      <c r="Q146" s="4">
         <v>1.3</v>
       </c>
     </row>
     <row r="147" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A147" t="s">
-        <v>17</v>
-      </c>
-      <c r="B147" t="s">
-        <v>18</v>
-      </c>
-      <c r="C147" t="s">
-        <v>19</v>
-      </c>
-      <c r="D147" t="s">
+      <c r="A147" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D147" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="E147">
+      <c r="E147" s="4">
         <v>374898</v>
       </c>
-      <c r="F147">
+      <c r="F147" s="4">
         <v>11687</v>
       </c>
-      <c r="G147">
+      <c r="G147" s="4">
         <v>17239.714</v>
       </c>
-      <c r="H147">
+      <c r="H147" s="4">
         <v>23473</v>
       </c>
-      <c r="I147">
+      <c r="I147" s="4">
         <v>807</v>
       </c>
-      <c r="J147">
+      <c r="J147" s="4">
         <v>954.42899999999997</v>
       </c>
-      <c r="K147">
+      <c r="K147" s="4">
         <v>1741.173</v>
       </c>
-      <c r="L147">
+      <c r="L147" s="4">
         <v>54.279000000000003</v>
       </c>
-      <c r="M147">
+      <c r="M147" s="4">
         <v>80.067999999999998</v>
       </c>
-      <c r="N147">
+      <c r="N147" s="4">
         <v>109.018</v>
       </c>
-      <c r="O147">
+      <c r="O147" s="4">
         <v>3.7480000000000002</v>
       </c>
-      <c r="P147">
+      <c r="P147" s="4">
         <v>4.4329999999999998</v>
       </c>
-      <c r="Q147">
+      <c r="Q147" s="4">
         <v>1.29</v>
       </c>
     </row>
     <row r="148" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
-        <v>17</v>
-      </c>
-      <c r="B148" t="s">
-        <v>18</v>
-      </c>
-      <c r="C148" t="s">
-        <v>19</v>
-      </c>
-      <c r="D148" t="s">
+      <c r="A148" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D148" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E148">
+      <c r="E148" s="4">
         <v>391222</v>
       </c>
-      <c r="F148">
+      <c r="F148" s="4">
         <v>16324</v>
       </c>
-      <c r="G148">
+      <c r="G148" s="4">
         <v>17084.857</v>
       </c>
-      <c r="H148">
+      <c r="H148" s="4">
         <v>24512</v>
       </c>
-      <c r="I148">
+      <c r="I148" s="4">
         <v>1039</v>
       </c>
-      <c r="J148">
+      <c r="J148" s="4">
         <v>934.42899999999997</v>
       </c>
-      <c r="K148">
+      <c r="K148" s="4">
         <v>1816.9880000000001</v>
       </c>
-      <c r="L148">
+      <c r="L148" s="4">
         <v>75.814999999999998</v>
       </c>
-      <c r="M148">
+      <c r="M148" s="4">
         <v>79.349000000000004</v>
       </c>
-      <c r="N148">
+      <c r="N148" s="4">
         <v>113.843</v>
       </c>
-      <c r="O148">
+      <c r="O148" s="4">
         <v>4.8259999999999996</v>
       </c>
-      <c r="P148">
+      <c r="P148" s="4">
         <v>4.34</v>
       </c>
-      <c r="Q148">
+      <c r="Q148" s="4">
         <v>1.29</v>
       </c>
     </row>
     <row r="149" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A149" t="s">
-        <v>17</v>
-      </c>
-      <c r="B149" t="s">
-        <v>18</v>
-      </c>
-      <c r="C149" t="s">
-        <v>19</v>
-      </c>
-      <c r="D149" t="s">
+      <c r="A149" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D149" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="E149">
+      <c r="E149" s="4">
         <v>411821</v>
       </c>
-      <c r="F149">
+      <c r="F149" s="4">
         <v>20599</v>
       </c>
-      <c r="G149">
+      <c r="G149" s="4">
         <v>17177.429</v>
       </c>
-      <c r="H149">
+      <c r="H149" s="4">
         <v>25598</v>
       </c>
-      <c r="I149">
+      <c r="I149" s="4">
         <v>1086</v>
       </c>
-      <c r="J149">
+      <c r="J149" s="4">
         <v>962.71400000000006</v>
       </c>
-      <c r="K149">
+      <c r="K149" s="4">
         <v>1912.6579999999999</v>
       </c>
-      <c r="L149">
+      <c r="L149" s="4">
         <v>95.67</v>
       </c>
-      <c r="M149">
+      <c r="M149" s="4">
         <v>79.778999999999996</v>
       </c>
-      <c r="N149">
+      <c r="N149" s="4">
         <v>118.887</v>
       </c>
-      <c r="O149">
+      <c r="O149" s="4">
         <v>5.0439999999999996</v>
       </c>
-      <c r="P149">
+      <c r="P149" s="4">
         <v>4.4710000000000001</v>
       </c>
-      <c r="Q149">
+      <c r="Q149" s="4">
         <v>1.28</v>
       </c>
     </row>
     <row r="150" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A150" t="s">
-        <v>17</v>
-      </c>
-      <c r="B150" t="s">
-        <v>18</v>
-      </c>
-      <c r="C150" t="s">
-        <v>19</v>
-      </c>
-      <c r="D150" t="s">
+      <c r="A150" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D150" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="E150">
+      <c r="E150" s="4">
         <v>438238</v>
       </c>
-      <c r="F150">
+      <c r="F150" s="4">
         <v>26417</v>
       </c>
-      <c r="G150">
+      <c r="G150" s="4">
         <v>18307.286</v>
       </c>
-      <c r="H150">
+      <c r="H150" s="4">
         <v>26754</v>
       </c>
-      <c r="I150">
+      <c r="I150" s="4">
         <v>1156</v>
       </c>
-      <c r="J150">
+      <c r="J150" s="4">
         <v>958.14300000000003</v>
       </c>
-      <c r="K150">
+      <c r="K150" s="4">
         <v>2035.348</v>
       </c>
-      <c r="L150">
+      <c r="L150" s="4">
         <v>122.691</v>
       </c>
-      <c r="M150">
+      <c r="M150" s="4">
         <v>85.025999999999996</v>
       </c>
-      <c r="N150">
+      <c r="N150" s="4">
         <v>124.256</v>
       </c>
-      <c r="O150">
+      <c r="O150" s="4">
         <v>5.3689999999999998</v>
       </c>
-      <c r="P150">
+      <c r="P150" s="4">
         <v>4.45</v>
       </c>
-      <c r="Q150">
+      <c r="Q150" s="4">
         <v>1.28</v>
       </c>
     </row>
     <row r="151" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A151" t="s">
-        <v>17</v>
-      </c>
-      <c r="B151" t="s">
-        <v>18</v>
-      </c>
-      <c r="C151" t="s">
-        <v>19</v>
-      </c>
-      <c r="D151" t="s">
+      <c r="A151" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C151" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D151" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="E151">
+      <c r="E151" s="4">
         <v>465166</v>
       </c>
-      <c r="F151">
+      <c r="F151" s="4">
         <v>26928</v>
       </c>
-      <c r="G151">
+      <c r="G151" s="4">
         <v>19182.286</v>
       </c>
-      <c r="H151">
+      <c r="H151" s="4">
         <v>27878</v>
       </c>
-      <c r="I151">
+      <c r="I151" s="4">
         <v>1124</v>
       </c>
-      <c r="J151">
+      <c r="J151" s="4">
         <v>975.71400000000006</v>
       </c>
-      <c r="K151">
+      <c r="K151" s="4">
         <v>2160.413</v>
       </c>
-      <c r="L151">
+      <c r="L151" s="4">
         <v>125.06399999999999</v>
       </c>
-      <c r="M151">
+      <c r="M151" s="4">
         <v>89.09</v>
       </c>
-      <c r="N151">
+      <c r="N151" s="4">
         <v>129.476</v>
       </c>
-      <c r="O151">
+      <c r="O151" s="4">
         <v>5.22</v>
       </c>
-      <c r="P151">
+      <c r="P151" s="4">
         <v>4.532</v>
       </c>
-      <c r="Q151">
+      <c r="Q151" s="4">
         <v>1.27</v>
       </c>
     </row>
     <row r="152" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A152" t="s">
-        <v>17</v>
-      </c>
-      <c r="B152" t="s">
-        <v>18</v>
-      </c>
-      <c r="C152" t="s">
-        <v>19</v>
-      </c>
-      <c r="D152" t="s">
+      <c r="A152" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D152" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E152">
+      <c r="E152" s="3">
         <v>498440</v>
       </c>
-      <c r="F152">
+      <c r="F152" s="3">
         <v>33274</v>
       </c>
-      <c r="G152">
+      <c r="G152" s="3">
         <v>21577.429</v>
       </c>
-      <c r="H152">
+      <c r="H152" s="3">
         <v>28834</v>
       </c>
-      <c r="I152">
+      <c r="I152" s="3">
         <v>956</v>
       </c>
-      <c r="J152">
+      <c r="J152" s="3">
         <v>974.42899999999997</v>
       </c>
-      <c r="K152">
+      <c r="K152" s="3">
         <v>2314.9499999999998</v>
       </c>
-      <c r="L152">
+      <c r="L152" s="3">
         <v>154.53700000000001</v>
       </c>
-      <c r="M152">
+      <c r="M152" s="3">
         <v>100.214</v>
       </c>
-      <c r="N152">
+      <c r="N152" s="3">
         <v>133.916</v>
       </c>
-      <c r="O152">
+      <c r="O152" s="3">
         <v>4.4400000000000004</v>
       </c>
-      <c r="P152">
+      <c r="P152" s="3">
         <v>4.5259999999999998</v>
       </c>
-      <c r="Q152">
+      <c r="Q152" s="3">
         <v>1.26</v>
       </c>
     </row>
     <row r="153" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A153" t="s">
-        <v>17</v>
-      </c>
-      <c r="B153" t="s">
-        <v>18</v>
-      </c>
-      <c r="C153" t="s">
-        <v>19</v>
-      </c>
-      <c r="D153" t="s">
+      <c r="A153" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D153" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="E153">
+      <c r="E153" s="3">
         <v>514849</v>
       </c>
-      <c r="F153">
+      <c r="F153" s="3">
         <v>16409</v>
       </c>
-      <c r="G153">
+      <c r="G153" s="3">
         <v>21662.571</v>
       </c>
-      <c r="H153">
+      <c r="H153" s="3">
         <v>29314</v>
       </c>
-      <c r="I153">
+      <c r="I153" s="3">
         <v>480</v>
       </c>
-      <c r="J153">
+      <c r="J153" s="3">
         <v>949.71400000000006</v>
       </c>
-      <c r="K153">
+      <c r="K153" s="3">
         <v>2391.16</v>
       </c>
-      <c r="L153">
+      <c r="L153" s="3">
         <v>76.209999999999994</v>
       </c>
-      <c r="M153">
+      <c r="M153" s="3">
         <v>100.60899999999999</v>
       </c>
-      <c r="N153">
+      <c r="N153" s="3">
         <v>136.14599999999999</v>
       </c>
-      <c r="O153">
+      <c r="O153" s="3">
         <v>2.2290000000000001</v>
       </c>
-      <c r="P153">
+      <c r="P153" s="3">
         <v>4.4109999999999996</v>
       </c>
-      <c r="Q153">
+      <c r="Q153" s="3">
         <v>1.25</v>
       </c>
     </row>
     <row r="154" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A154" t="s">
-        <v>17</v>
-      </c>
-      <c r="B154" t="s">
-        <v>18</v>
-      </c>
-      <c r="C154" t="s">
-        <v>19</v>
-      </c>
-      <c r="D154" t="s">
+      <c r="A154" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D154" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E154">
+      <c r="E154" s="3">
         <v>526447</v>
       </c>
-      <c r="F154">
+      <c r="F154" s="3">
         <v>11598</v>
       </c>
-      <c r="G154">
+      <c r="G154" s="3">
         <v>21649.857</v>
       </c>
-      <c r="H154">
+      <c r="H154" s="3">
         <v>29937</v>
       </c>
-      <c r="I154">
+      <c r="I154" s="3">
         <v>623</v>
       </c>
-      <c r="J154">
+      <c r="J154" s="3">
         <v>923.42899999999997</v>
       </c>
-      <c r="K154">
+      <c r="K154" s="3">
         <v>2445.0250000000001</v>
       </c>
-      <c r="L154">
+      <c r="L154" s="3">
         <v>53.866</v>
       </c>
-      <c r="M154">
+      <c r="M154" s="3">
         <v>100.55</v>
       </c>
-      <c r="N154">
+      <c r="N154" s="3">
         <v>139.03899999999999</v>
       </c>
-      <c r="O154">
+      <c r="O154" s="3">
         <v>2.8929999999999998</v>
       </c>
-      <c r="P154">
+      <c r="P154" s="3">
         <v>4.2889999999999997</v>
       </c>
-      <c r="Q154">
+      <c r="Q154" s="3">
         <v>1.24</v>
       </c>
     </row>
     <row r="155" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A155" t="s">
-        <v>17</v>
-      </c>
-      <c r="B155" t="s">
-        <v>18</v>
-      </c>
-      <c r="C155" t="s">
-        <v>19</v>
-      </c>
-      <c r="D155" t="s">
+      <c r="A155" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C155" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D155" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E155">
+      <c r="E155" s="3">
         <v>555383</v>
       </c>
-      <c r="F155">
+      <c r="F155" s="3">
         <v>28936</v>
       </c>
-      <c r="G155">
+      <c r="G155" s="3">
         <v>23451.571</v>
       </c>
-      <c r="H155">
+      <c r="H155" s="3">
         <v>31199</v>
       </c>
-      <c r="I155">
+      <c r="I155" s="3">
         <v>1262</v>
       </c>
-      <c r="J155">
+      <c r="J155" s="3">
         <v>955.28599999999994</v>
       </c>
-      <c r="K155">
+      <c r="K155" s="3">
         <v>2579.4160000000002</v>
       </c>
-      <c r="L155">
+      <c r="L155" s="3">
         <v>134.38999999999999</v>
       </c>
-      <c r="M155">
+      <c r="M155" s="3">
         <v>108.91800000000001</v>
       </c>
-      <c r="N155">
+      <c r="N155" s="3">
         <v>144.9</v>
       </c>
-      <c r="O155">
+      <c r="O155" s="3">
         <v>5.8609999999999998</v>
       </c>
-      <c r="P155">
+      <c r="P155" s="3">
         <v>4.4370000000000003</v>
       </c>
-      <c r="Q155">
+      <c r="Q155" s="3">
         <v>1.23</v>
       </c>
     </row>
     <row r="156" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A156" t="s">
-        <v>17</v>
-      </c>
-      <c r="B156" t="s">
-        <v>18</v>
-      </c>
-      <c r="C156" t="s">
-        <v>19</v>
-      </c>
-      <c r="D156" t="s">
+      <c r="A156" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D156" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E156">
+      <c r="E156" s="3">
         <v>584016</v>
       </c>
-      <c r="F156">
+      <c r="F156" s="3">
         <v>28633</v>
       </c>
-      <c r="G156">
+      <c r="G156" s="3">
         <v>24599.286</v>
       </c>
-      <c r="H156">
+      <c r="H156" s="3">
         <v>32548</v>
       </c>
-      <c r="I156">
+      <c r="I156" s="3">
         <v>1349</v>
       </c>
-      <c r="J156">
+      <c r="J156" s="3">
         <v>992.85699999999997</v>
       </c>
-      <c r="K156">
+      <c r="K156" s="3">
         <v>2712.3980000000001</v>
       </c>
-      <c r="L156">
+      <c r="L156" s="3">
         <v>132.983</v>
       </c>
-      <c r="M156">
+      <c r="M156" s="3">
         <v>114.249</v>
       </c>
-      <c r="N156">
+      <c r="N156" s="3">
         <v>151.166</v>
       </c>
-      <c r="O156">
+      <c r="O156" s="3">
         <v>6.2649999999999997</v>
       </c>
-      <c r="P156">
+      <c r="P156" s="3">
         <v>4.6109999999999998</v>
       </c>
-      <c r="Q156">
+      <c r="Q156" s="3">
         <v>1.22</v>
       </c>
     </row>
     <row r="157" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A157" t="s">
-        <v>17</v>
-      </c>
-      <c r="B157" t="s">
-        <v>18</v>
-      </c>
-      <c r="C157" t="s">
-        <v>19</v>
-      </c>
-      <c r="D157" t="s">
+      <c r="A157" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D157" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E157">
+      <c r="E157" s="3">
         <v>614941</v>
       </c>
-      <c r="F157">
+      <c r="F157" s="3">
         <v>30925</v>
       </c>
-      <c r="G157">
+      <c r="G157" s="3">
         <v>25243.286</v>
       </c>
-      <c r="H157">
+      <c r="H157" s="3">
         <v>34021</v>
       </c>
-      <c r="I157">
+      <c r="I157" s="3">
         <v>1473</v>
       </c>
-      <c r="J157">
+      <c r="J157" s="3">
         <v>1038.143</v>
       </c>
-      <c r="K157">
+      <c r="K157" s="3">
         <v>2856.0259999999998</v>
       </c>
-      <c r="L157">
+      <c r="L157" s="3">
         <v>143.62799999999999</v>
       </c>
-      <c r="M157">
+      <c r="M157" s="3">
         <v>117.24</v>
       </c>
-      <c r="N157">
+      <c r="N157" s="3">
         <v>158.00700000000001</v>
       </c>
-      <c r="O157">
+      <c r="O157" s="3">
         <v>6.8410000000000002</v>
       </c>
-      <c r="P157">
+      <c r="P157" s="3">
         <v>4.8220000000000001</v>
       </c>
-      <c r="Q157">
+      <c r="Q157" s="3">
         <v>1.22</v>
       </c>
     </row>
     <row r="158" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A158" t="s">
-        <v>17</v>
-      </c>
-      <c r="B158" t="s">
-        <v>18</v>
-      </c>
-      <c r="C158" t="s">
-        <v>19</v>
-      </c>
-      <c r="D158" t="s">
+      <c r="A158" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D158" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E158">
+      <c r="E158" s="3">
         <v>645771</v>
       </c>
-      <c r="F158">
+      <c r="F158" s="3">
         <v>30830</v>
       </c>
-      <c r="G158">
+      <c r="G158" s="3">
         <v>25800.714</v>
       </c>
-      <c r="H158">
+      <c r="H158" s="3">
         <v>35026</v>
       </c>
-      <c r="I158">
+      <c r="I158" s="3">
         <v>1005</v>
       </c>
-      <c r="J158">
+      <c r="J158" s="3">
         <v>1021.143</v>
       </c>
-      <c r="K158">
+      <c r="K158" s="3">
         <v>2999.2130000000002</v>
       </c>
-      <c r="L158">
+      <c r="L158" s="3">
         <v>143.18700000000001</v>
       </c>
-      <c r="M158">
+      <c r="M158" s="3">
         <v>119.82899999999999</v>
       </c>
-      <c r="N158">
+      <c r="N158" s="3">
         <v>162.67400000000001</v>
       </c>
-      <c r="O158">
+      <c r="O158" s="3">
         <v>4.6680000000000001</v>
       </c>
-      <c r="P158">
+      <c r="P158" s="3">
         <v>4.7430000000000003</v>
       </c>
-      <c r="Q158">
+      <c r="Q158" s="3">
         <v>1.21</v>
       </c>
     </row>
     <row r="159" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A159" t="s">
-        <v>17</v>
-      </c>
-      <c r="B159" t="s">
-        <v>18</v>
-      </c>
-      <c r="C159" t="s">
-        <v>19</v>
-      </c>
-      <c r="D159" t="s">
+      <c r="A159" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D159" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E159">
+      <c r="E159" s="3">
         <v>672846</v>
       </c>
-      <c r="F159">
+      <c r="F159" s="3">
         <v>27075</v>
       </c>
-      <c r="G159">
+      <c r="G159" s="3">
         <v>24915.143</v>
       </c>
-      <c r="H159">
+      <c r="H159" s="3">
         <v>35930</v>
       </c>
-      <c r="I159">
+      <c r="I159" s="3">
         <v>904</v>
       </c>
-      <c r="J159">
+      <c r="J159" s="3">
         <v>1013.7140000000001</v>
       </c>
-      <c r="K159">
+      <c r="K159" s="3">
         <v>3124.96</v>
       </c>
-      <c r="L159">
+      <c r="L159" s="3">
         <v>125.747</v>
       </c>
-      <c r="M159">
+      <c r="M159" s="3">
         <v>115.71599999999999</v>
       </c>
-      <c r="N159">
+      <c r="N159" s="3">
         <v>166.87299999999999</v>
       </c>
-      <c r="O159">
+      <c r="O159" s="3">
         <v>4.1989999999999998</v>
       </c>
-      <c r="P159">
+      <c r="P159" s="3">
         <v>4.7080000000000002</v>
       </c>
-      <c r="Q159">
+      <c r="Q159" s="3">
         <v>1.2</v>
       </c>
     </row>
     <row r="160" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A160" t="s">
-        <v>17</v>
-      </c>
-      <c r="B160" t="s">
-        <v>18</v>
-      </c>
-      <c r="C160" t="s">
-        <v>19</v>
-      </c>
-      <c r="D160" t="s">
+      <c r="A160" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D160" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E160">
+      <c r="E160" s="3">
         <v>691758</v>
       </c>
-      <c r="F160">
+      <c r="F160" s="3">
         <v>18912</v>
       </c>
-      <c r="G160">
+      <c r="G160" s="3">
         <v>25272.714</v>
       </c>
-      <c r="H160">
+      <c r="H160" s="3">
         <v>36455</v>
       </c>
-      <c r="I160">
+      <c r="I160" s="3">
         <v>525</v>
       </c>
-      <c r="J160">
+      <c r="J160" s="3">
         <v>1020.143</v>
       </c>
-      <c r="K160">
+      <c r="K160" s="3">
         <v>3212.7939999999999</v>
       </c>
-      <c r="L160">
+      <c r="L160" s="3">
         <v>87.834999999999994</v>
       </c>
-      <c r="M160">
+      <c r="M160" s="3">
         <v>117.376</v>
       </c>
-      <c r="N160">
+      <c r="N160" s="3">
         <v>169.31100000000001</v>
       </c>
-      <c r="O160">
+      <c r="O160" s="3">
         <v>2.4380000000000002</v>
       </c>
-      <c r="P160">
+      <c r="P160" s="3">
         <v>4.7380000000000004</v>
       </c>
-      <c r="Q160">
+      <c r="Q160" s="3">
         <v>1.2</v>
       </c>
     </row>
@@ -74366,7 +74382,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>

</xml_diff>